<commit_message>
feat: theme categories (macro/tech/politics/other/bbg-tv-news), fix YouTube dates, add Bloomberg TV + Citadel sources
</commit_message>
<xml_diff>
--- a/Buyside_research_list.xlsx
+++ b/Buyside_research_list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -234,6 +234,33 @@
   </si>
   <si>
     <t>https://hk.allianzgi.com/en-hk/retail/insights/insights-and-strategies</t>
+  </si>
+  <si>
+    <t>Wall Street Breakfast</t>
+  </si>
+  <si>
+    <t>https://seekingalpha.com/author/wall-street-breakfast</t>
+  </si>
+  <si>
+    <t>Citadel Insight</t>
+  </si>
+  <si>
+    <t>https://www.citadelsecurities.com/news-and-insights/category/market-insights/</t>
+  </si>
+  <si>
+    <t>Bloomberg TV</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/@markets</t>
+  </si>
+  <si>
+    <t>Bloomberg Podcasts</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/bloombergpodcasts</t>
+  </si>
+  <si>
+    <t>https://podcasts.apple.com/us/channel/bloomberg/id6442484579</t>
   </si>
 </sst>
 </file>
@@ -283,18 +310,13 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -321,9 +343,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1018,9 +1037,13 @@
       <c r="H33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="9"/>
+      <c r="A34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="4"/>
@@ -1028,8 +1051,12 @@
       <c r="H34" s="2"/>
     </row>
     <row r="35">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
+      <c r="A35" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -1038,8 +1065,12 @@
       <c r="H35" s="2"/>
     </row>
     <row r="36">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
+      <c r="A36" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -1048,8 +1079,12 @@
       <c r="H36" s="2"/>
     </row>
     <row r="37">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
+      <c r="A37" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>72</v>
+      </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -1058,8 +1093,12 @@
       <c r="H37" s="2"/>
     </row>
     <row r="38">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
+      <c r="A38" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>73</v>
+      </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -1088,60 +1127,60 @@
       <c r="H40" s="2"/>
     </row>
     <row r="41">
-      <c r="C41" s="10"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
     </row>
     <row r="42">
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
     </row>
     <row r="43">
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
     </row>
     <row r="44">
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
     </row>
     <row r="45">
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="11"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
     </row>
     <row r="46">
-      <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
     </row>
     <row r="47">
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
     </row>
     <row r="48">
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
     </row>
     <row r="49">
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
     </row>
     <row r="50">
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
     </row>
     <row r="51">
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="11"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1177,7 +1216,12 @@
     <hyperlink r:id="rId30" ref="B31"/>
     <hyperlink r:id="rId31" ref="B32"/>
     <hyperlink r:id="rId32" ref="B33"/>
+    <hyperlink r:id="rId33" ref="B34"/>
+    <hyperlink r:id="rId34" ref="B35"/>
+    <hyperlink r:id="rId35" ref="B36"/>
+    <hyperlink r:id="rId36" ref="B37"/>
+    <hyperlink r:id="rId37" ref="B38"/>
   </hyperlinks>
-  <drawing r:id="rId33"/>
+  <drawing r:id="rId38"/>
 </worksheet>
 </file>
</xml_diff>